<commit_message>
flujo de factura y  nota de credito con los 4 pasos del flujo
</commit_message>
<xml_diff>
--- a/tests/test_data/factura/factura_casos.xlsx
+++ b/tests/test_data/factura/factura_casos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ErickAlejandroRodríg\Desktop\Entorno\Auto FACTO 8\automation_framework\tests\test_data\factura\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF12EFA-FC0B-40AA-93E0-5C5397D91E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36A9662-8846-455A-B3C6-5C022DB7D652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factura" sheetId="1" r:id="rId1"/>
@@ -175,6 +175,9 @@
     <t>PUBLICO EN GENERAL</t>
   </si>
   <si>
+    <t>03104</t>
+  </si>
+  <si>
     <t>616 - Sin obligaciones fiscales</t>
   </si>
   <si>
@@ -242,16 +245,13 @@
   </si>
   <si>
     <t xml:space="preserve">002 - IVA </t>
-  </si>
-  <si>
-    <t>´03104</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -259,13 +259,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1760D7"/>
+        <bgColor rgb="FF1760D7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -280,8 +292,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -611,145 +627,151 @@
     <col min="32" max="32" width="14.7265625" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="21.6328125" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="15" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.1796875" customWidth="1"/>
+    <col min="36" max="36" width="18.7265625" customWidth="1"/>
+    <col min="39" max="39" width="13.90625" customWidth="1"/>
+    <col min="40" max="40" width="14.08984375" customWidth="1"/>
     <col min="41" max="41" width="26.1796875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="32" customWidth="1"/>
+    <col min="43" max="43" width="15.6328125" customWidth="1"/>
+    <col min="44" max="44" width="16.81640625" customWidth="1"/>
     <col min="45" max="45" width="18.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:45" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -772,80 +794,80 @@
       <c r="G2" t="s">
         <v>50</v>
       </c>
-      <c r="H2" t="s">
-        <v>74</v>
+      <c r="H2" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="I2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="S2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="T2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="U2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="V2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="W2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="X2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD2" t="s">
         <v>58</v>
       </c>
-      <c r="Y2" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>57</v>
-      </c>
       <c r="AE2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="AF2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="AG2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="AH2">
         <v>10</v>
       </c>
       <c r="AI2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AJ2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AK2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AL2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AM2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AN2">
         <v>16</v>
@@ -857,7 +879,7 @@
         <v>45</v>
       </c>
       <c r="AS2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: refactor cfdi flow + ajustes nota credito + outputs
</commit_message>
<xml_diff>
--- a/tests/test_data/factura/factura_casos.xlsx
+++ b/tests/test_data/factura/factura_casos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ErickAlejandroRodríg\Desktop\Entorno\Auto FACTO 8\automation_framework\tests\test_data\factura\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36A9662-8846-455A-B3C6-5C022DB7D652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3A1EF1-D5D2-4BA8-806B-9E1B53FD85C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factura" sheetId="1" r:id="rId1"/>
@@ -172,9 +172,6 @@
     <t>XAXX010101000</t>
   </si>
   <si>
-    <t>PUBLICO EN GENERAL</t>
-  </si>
-  <si>
     <t>03104</t>
   </si>
   <si>
@@ -245,6 +242,9 @@
   </si>
   <si>
     <t xml:space="preserve">002 - IVA </t>
+  </si>
+  <si>
+    <t>CFDI PUBLICO GENERAL</t>
   </si>
 </sst>
 </file>
@@ -792,82 +792,82 @@
         <v>49</v>
       </c>
       <c r="G2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" t="s">
         <v>51</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>52</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>53</v>
       </c>
-      <c r="K2" t="s">
+      <c r="R2" t="s">
         <v>54</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>55</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>56</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>57</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
+        <v>68</v>
+      </c>
+      <c r="W2" t="s">
+        <v>69</v>
+      </c>
+      <c r="X2" t="s">
         <v>58</v>
       </c>
-      <c r="V2" t="s">
-        <v>69</v>
-      </c>
-      <c r="W2" t="s">
+      <c r="Y2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC2" t="s">
         <v>70</v>
       </c>
-      <c r="X2" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB2" t="s">
+      <c r="AD2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE2" t="s">
         <v>62</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AF2" t="s">
         <v>71</v>
       </c>
-      <c r="AD2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>63</v>
-      </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>72</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>73</v>
       </c>
       <c r="AH2">
         <v>10</v>
       </c>
       <c r="AI2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ2" t="s">
         <v>64</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AK2" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL2" t="s">
         <v>65</v>
       </c>
-      <c r="AK2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AL2" t="s">
+      <c r="AM2" t="s">
         <v>66</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>67</v>
       </c>
       <c r="AN2">
         <v>16</v>
@@ -879,7 +879,7 @@
         <v>45</v>
       </c>
       <c r="AS2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Flujo FACUTRA NOTA DE CREDITO PPD done
</commit_message>
<xml_diff>
--- a/tests/test_data/factura/factura_casos.xlsx
+++ b/tests/test_data/factura/factura_casos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ErickAlejandroRodríg\Desktop\Entorno\Auto FACTO 8\automation_framework\tests\test_data\factura\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3A1EF1-D5D2-4BA8-806B-9E1B53FD85C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD623B9-4E04-46C7-BB9E-9C4E7F695CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factura" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="74">
   <si>
     <t>ejecutar</t>
   </si>
@@ -182,9 +182,6 @@
   </si>
   <si>
     <t>alejandro.rodriguez@next-technologies.com.mx</t>
-  </si>
-  <si>
-    <t>AUTO</t>
   </si>
   <si>
     <t>01 - No aplica</t>
@@ -292,12 +289,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -613,7 +611,7 @@
     <col min="9" max="9" width="26" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.54296875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="42.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="12.08984375" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="19.36328125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="11.453125" bestFit="1" customWidth="1"/>
@@ -792,7 +790,7 @@
         <v>49</v>
       </c>
       <c r="G2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>50</v>
@@ -806,68 +804,68 @@
       <c r="K2" t="s">
         <v>53</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="3">
+        <v>46141.465752314813</v>
+      </c>
+      <c r="S2" t="s">
         <v>54</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>55</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>56</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
+        <v>67</v>
+      </c>
+      <c r="W2" t="s">
+        <v>68</v>
+      </c>
+      <c r="X2" t="s">
         <v>57</v>
       </c>
-      <c r="V2" t="s">
-        <v>68</v>
-      </c>
-      <c r="W2" t="s">
+      <c r="Y2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC2" t="s">
         <v>69</v>
       </c>
-      <c r="X2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB2" t="s">
+      <c r="AD2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE2" t="s">
         <v>61</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AF2" t="s">
         <v>70</v>
       </c>
-      <c r="AD2" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>62</v>
-      </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>71</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>72</v>
       </c>
       <c r="AH2">
         <v>10</v>
       </c>
       <c r="AI2" t="s">
+        <v>62</v>
+      </c>
+      <c r="AJ2" t="s">
         <v>63</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AK2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AL2" t="s">
         <v>64</v>
       </c>
-      <c r="AK2" t="s">
-        <v>73</v>
-      </c>
-      <c r="AL2" t="s">
+      <c r="AM2" t="s">
         <v>65</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>66</v>
       </c>
       <c r="AN2">
         <v>16</v>
@@ -879,7 +877,7 @@
         <v>45</v>
       </c>
       <c r="AS2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>